<commit_message>
Brand Control Kit app and Excel export in black and yellow
</commit_message>
<xml_diff>
--- a/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -22,45 +22,51 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF202326"/>
+      <color rgb="FF09090B"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF202326"/>
+      <color rgb="FF09090B"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFFC700"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFFC700"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFF4F4F5"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF175CD3"/>
+      <color rgb="FF725800"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF6B7280"/>
+      <color rgb="FF71717A"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFFFC700"/>
     </font>
   </fonts>
   <fills count="11">
@@ -78,13 +84,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F4F7"/>
+        <fgColor rgb="FFF4F4F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF13294B"/>
+        <fgColor rgb="FF09090B"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -102,25 +108,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2B705"/>
+        <fgColor rgb="FFFFC700"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6B7280"/>
+        <fgColor rgb="FF71717A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6D28D9"/>
+        <fgColor rgb="FF26262C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3EFFF"/>
+        <fgColor rgb="FFFFF8D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -146,12 +152,12 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
@@ -165,15 +171,53 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="952500" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Control Kit logo" descr="Black and yellow Control Kit hexagon logo"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -199,10 +243,10 @@
     <col min="13" max="13" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control Kit — Bill of Materials</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
@@ -212,7 +256,7 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">CONTROL KIT  /  BILL OF MATERIALS</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
@@ -266,22 +310,22 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Assembly: FTC Competition Robot · Open in Onshape</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
@@ -333,20 +377,20 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Generated: 10/23/2026, 8:00:00 AM · Vendor data as of: 2026-10-23T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -929,16 +973,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:M10"/>
-  <mergeCells count="6">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:M1"/>
+    <mergeCell ref="C2:M2"/>
+    <mergeCell ref="C3:M3"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A12:M12"/>
     <mergeCell ref="A16:M16"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="C2" r:id="rId1"/>
     <hyperlink ref="E7" r:id="rId2"/>
     <hyperlink ref="E8" r:id="rId3"/>
     <hyperlink ref="E9" r:id="rId4"/>
@@ -951,6 +996,7 @@
   <printOptions/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Match Control Kit branding across app and Excel BOM (#8)
* Brand Control Kit app and Excel export in black and yellow

* Keep Excel export available when logo asset fails

* Await Excel fallback assertion in browser test
</commit_message>
<xml_diff>
--- a/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -22,45 +22,51 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF202326"/>
+      <color rgb="FF09090B"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF202326"/>
+      <color rgb="FF09090B"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFFC700"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFFC700"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFF4F4F5"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF175CD3"/>
+      <color rgb="FF725800"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF6B7280"/>
+      <color rgb="FF71717A"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFFFC700"/>
     </font>
   </fonts>
   <fills count="11">
@@ -78,13 +84,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F4F7"/>
+        <fgColor rgb="FFF4F4F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF13294B"/>
+        <fgColor rgb="FF09090B"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -102,25 +108,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2B705"/>
+        <fgColor rgb="FFFFC700"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6B7280"/>
+        <fgColor rgb="FF71717A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6D28D9"/>
+        <fgColor rgb="FF26262C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3EFFF"/>
+        <fgColor rgb="FFFFF8D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -146,12 +152,12 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
@@ -165,15 +171,53 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="952500" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Control Kit logo" descr="Black and yellow Control Kit hexagon logo"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -199,10 +243,10 @@
     <col min="13" max="13" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control Kit — Bill of Materials</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
@@ -212,7 +256,7 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">CONTROL KIT  /  BILL OF MATERIALS</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
@@ -266,22 +310,22 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Assembly: FTC Competition Robot · Open in Onshape</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
@@ -333,20 +377,20 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Generated: 10/23/2026, 8:00:00 AM · Vendor data as of: 2026-10-23T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -929,16 +973,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:M10"/>
-  <mergeCells count="6">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:M1"/>
+    <mergeCell ref="C2:M2"/>
+    <mergeCell ref="C3:M3"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A12:M12"/>
     <mergeCell ref="A16:M16"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="C2" r:id="rId1"/>
     <hyperlink ref="E7" r:id="rId2"/>
     <hyperlink ref="E8" r:id="rId3"/>
     <hyperlink ref="E9" r:id="rId4"/>
@@ -951,6 +996,7 @@
   <printOptions/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Model how each part is obtained, with evidence and shared overrides
Replace the print keyword score with a disposition (Buy, 3D print, CNC,
2D cut, other fabrication, Needs review) decided by a fixed precedence:
manual choice, exact SKU, explicit metadata (BOM process column, team tags,
print material), strong provenance, then a reviewable suggestion. Exact-SKU
parts stay Buy unless a person overrides them, and that exception is shown.
Manual choices are shared per document with who set them and a short
history, require the writer's own scan of the document, and still honor
pre-rework per-user saves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -225,7 +225,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -238,7 +238,7 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="38" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
   </cols>
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="F4" s="22">
-        <f>SUM(H7:H13)</f>
+        <f>SUM(H7:H11)</f>
         <v>979.6</v>
       </c>
       <c r="G4" s="20" t="inlineStr">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="J4" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -600,7 +600,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commercial</t>
+          <t xml:space="preserve">Buy</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commercial</t>
+          <t xml:space="preserve">Buy</t>
         </is>
       </c>
       <c r="M8" s="1" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commercial</t>
+          <t xml:space="preserve">Buy</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commercial</t>
+          <t xml:space="preserve">Buy</t>
         </is>
       </c>
       <c r="M10" s="1" t="inlineStr">
@@ -755,232 +755,164 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">— 3D PRINTED PARTS —</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="L12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M12" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2">
+    <row r="11">
+      <c r="A11" s="0">
         <v>5</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Custom Printed Intake Guide</t>
         </is>
       </c>
-      <c r="C13" s="2">
+      <c r="C11" s="0">
         <v>10</v>
       </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3D Printed</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Print</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3D Printed</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs review</t>
+        </is>
+      </c>
+      <c r="M11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— IN-STOCK ALTERNATIVES —</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96mm Wheel</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rev</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REV-31-1240</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96mm Wheel — alternate hub — $13.25</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">— IN-STOCK ALTERNATIVES —</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="L16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M16" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="0" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">96mm Wheel</t>
         </is>
       </c>
-      <c r="E17" s="0" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">rev</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">REV-31-1240</t>
-        </is>
-      </c>
-      <c r="L17" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">96mm Wheel — alternate hub — $13.25</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">96mm Wheel</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rev</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">REV-31-1241</t>
         </is>
       </c>
-      <c r="L18" s="18" t="inlineStr">
+      <c r="L16" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">96mm Wheel — alternate tread — $14.50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M10"/>
-  <mergeCells count="7">
+  <autoFilter ref="A6:M11"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:M1"/>
     <mergeCell ref="C2:M2"/>
     <mergeCell ref="C3:M3"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A12:M12"/>
-    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A14:M14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1"/>
@@ -989,14 +921,13 @@
     <hyperlink ref="E9" r:id="rId4"/>
     <hyperlink ref="L9" r:id="rId5"/>
     <hyperlink ref="E10" r:id="rId6"/>
-    <hyperlink ref="E13" r:id="rId7"/>
-    <hyperlink ref="L17" r:id="rId8"/>
-    <hyperlink ref="L18" r:id="rId9"/>
+    <hyperlink ref="L15" r:id="rId7"/>
+    <hyperlink ref="L16" r:id="rId8"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
-  <drawing r:id="rId10"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -1005,12 +936,12 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,36 +979,11 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Printed Intake Guide</t>
-        </is>
-      </c>
-      <c r="B2" s="0">
-        <v>10</v>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">intake</t>
-        </is>
-      </c>
-      <c r="D2" s="0">
-        <v>100</v>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">strong print keyword (+50); keyword: custom (+20); keyword: guide (+20); no vendor or SKU-like number (+25)</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://cad.onshape.com/documents/robot/w/fixture/e/prints</t>
+          <t xml:space="preserve">No 3D printed parts detected.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-  </hyperlinks>
   <printOptions/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>

</xml_diff>

<commit_message>
Review holds unmatched Buy parts, the drawer moves on after a choice, and bulk types
Parts to buy with no vendor product now wait in Review (No product), with the
products, vendor search, and type changes that fix each; Review's count, the
primary action, and next moves count them. The part drawer moves to the next
part in the list it came from after a saved choice and says where the part went.
Review rows can be selected (shift-click range, whole subassembly) and given one
type, saved per part with failures kept selected. Pattern and Replicate copies
are already counted (the definition lists them as instances); a fixture pins it.
</commit_message>
<xml_diff>
--- a/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -214,10 +214,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -413,7 +413,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -758,9 +758,9 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
     <col min="14" max="14" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -911,7 +911,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1075,17 +1075,17 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Price and Stock As Of</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Match</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product</t>
-        </is>
-      </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -1098,7 +1098,7 @@
       <c r="A7" s="0">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">M3 Screw</t>
         </is>
@@ -1136,17 +1136,17 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L7" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L7" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N7" s="25" t="inlineStr">
@@ -1159,7 +1159,7 @@
       <c r="A8" s="1">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">5203 Motor</t>
         </is>
@@ -1197,17 +1197,17 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L8" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N8" s="26" t="inlineStr">
@@ -1220,7 +1220,7 @@
       <c r="A9" s="0">
         <v>3</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">96mm Wheel</t>
         </is>
@@ -1258,17 +1258,17 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L9" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N9" s="25" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="A10" s="1">
         <v>4</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Bearing</t>
         </is>
@@ -1324,17 +1324,17 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L10" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M10" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N10" s="26" t="inlineStr">
@@ -1353,13 +1353,13 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="L7" r:id="rId2"/>
+    <hyperlink ref="B7" r:id="rId2"/>
     <hyperlink ref="M7" r:id="rId3"/>
-    <hyperlink ref="L8" r:id="rId4"/>
+    <hyperlink ref="B8" r:id="rId4"/>
     <hyperlink ref="M8" r:id="rId5"/>
-    <hyperlink ref="L9" r:id="rId6"/>
+    <hyperlink ref="B9" r:id="rId6"/>
     <hyperlink ref="M9" r:id="rId7"/>
-    <hyperlink ref="L10" r:id="rId8"/>
+    <hyperlink ref="B10" r:id="rId8"/>
     <hyperlink ref="M10" r:id="rId9"/>
   </hyperlinks>
   <printOptions/>
@@ -1382,7 +1382,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1473,7 +1473,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="64" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1679,7 +1679,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1910,7 +1910,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="72" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2296,7 +2296,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -2376,12 +2376,12 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">REV REV-31-1234 as of 2026-10-23</t>
+          <t xml:space="preserve">REV REV-31-1234, as of 2026-10-23</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Review holds unmatched Buy parts, the drawer moves on after a choice, and bulk types (#59)
* Review holds unmatched Buy parts, the drawer moves on after a choice, and bulk types

Parts to buy with no vendor product now wait in Review (No product), with the
products, vendor search, and type changes that fix each; Review's count, the
primary action, and next moves count them. The part drawer moves to the next
part in the list it came from after a saved choice and says where the part went.
Review rows can be selected (shift-click range, whole subassembly) and given one
type, saved per part with failures kept selected. Pattern and Replicate copies
are already counted (the definition lists them as instances); a fixture pins it.

* Greptile: a bulk save skips parts changed while it waited; the drawer stays in its Review group

* Greptile: subassembly selection follows the path, not the name; shift-click anchors by part
</commit_message>
<xml_diff>
--- a/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/samples/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -214,10 +214,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -413,7 +413,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -758,9 +758,9 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
     <col min="14" max="14" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -911,7 +911,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1075,17 +1075,17 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Price and Stock As Of</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Match</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product</t>
-        </is>
-      </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -1098,7 +1098,7 @@
       <c r="A7" s="0">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">M3 Screw</t>
         </is>
@@ -1136,17 +1136,17 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L7" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L7" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N7" s="25" t="inlineStr">
@@ -1159,7 +1159,7 @@
       <c r="A8" s="1">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">5203 Motor</t>
         </is>
@@ -1197,17 +1197,17 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L8" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N8" s="26" t="inlineStr">
@@ -1220,7 +1220,7 @@
       <c r="A9" s="0">
         <v>3</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">96mm Wheel</t>
         </is>
@@ -1258,17 +1258,17 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L9" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N9" s="25" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="A10" s="1">
         <v>4</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Bearing</t>
         </is>
@@ -1324,17 +1324,17 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Confirmed</t>
         </is>
       </c>
-      <c r="L10" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product page</t>
-        </is>
-      </c>
       <c r="M10" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
       <c r="N10" s="26" t="inlineStr">
@@ -1353,13 +1353,13 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="L7" r:id="rId2"/>
+    <hyperlink ref="B7" r:id="rId2"/>
     <hyperlink ref="M7" r:id="rId3"/>
-    <hyperlink ref="L8" r:id="rId4"/>
+    <hyperlink ref="B8" r:id="rId4"/>
     <hyperlink ref="M8" r:id="rId5"/>
-    <hyperlink ref="L9" r:id="rId6"/>
+    <hyperlink ref="B9" r:id="rId6"/>
     <hyperlink ref="M9" r:id="rId7"/>
-    <hyperlink ref="L10" r:id="rId8"/>
+    <hyperlink ref="B10" r:id="rId8"/>
     <hyperlink ref="M10" r:id="rId9"/>
   </hyperlinks>
   <printOptions/>
@@ -1382,7 +1382,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1473,7 +1473,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="64" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1679,7 +1679,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1910,7 +1910,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="72" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2296,7 +2296,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanned 2026-10-24 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
+          <t xml:space="preserve">Scanned 2026-10-29 (Not recorded) · Generated 2026-10-23 12:00 UTC</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Onshape part</t>
+          <t xml:space="preserve">Onshape Part Studio</t>
         </is>
       </c>
     </row>
@@ -2376,12 +2376,12 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">REV REV-31-1234 as of 2026-10-23</t>
+          <t xml:space="preserve">REV REV-31-1234, as of 2026-10-23</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open in Onshape</t>
+          <t xml:space="preserve">Open Part Studio</t>
         </is>
       </c>
     </row>

</xml_diff>